<commit_message>
Indiegogo draft and financial model fix
</commit_message>
<xml_diff>
--- a/docs/civicview_financial_model.xlsx
+++ b/docs/civicview_financial_model.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
@@ -30,8 +30,9 @@
     <numFmt numFmtId="168" formatCode="0.0&quot; months&quot;"/>
     <numFmt numFmtId="169" formatCode="$#,##0.00"/>
     <numFmt numFmtId="170" formatCode="$#,##0"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -286,6 +287,17 @@
     <font>
       <color rgb="001F4E79"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF5F5E5A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -335,7 +347,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -677,6 +689,11 @@
     <xf numFmtId="166" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
+    <xf numFmtId="171" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1140,7 +1157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="59" min="1" max="1"/>
@@ -1891,7 +1908,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="59" t="inlineStr">
         <is>
           <t>Google Workspace Business Starter (annual)</t>
         </is>
@@ -1900,14 +1917,14 @@
         <f>8.4*12</f>
         <v/>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="59" t="inlineStr">
         <is>
           <t>$8.40/mo x 12 = $100.80/yr. Custom domain email + Drive/Docs for the founder.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="59" t="inlineStr">
         <is>
           <t>Vote Smart API license — OPTIONAL toggle (1 = include, 0 = exclude)</t>
         </is>
@@ -1915,14 +1932,14 @@
       <c r="B64" s="97" t="n">
         <v>0</v>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="59" t="inlineStr">
         <is>
           <t>Set to 1 to include the Vote Smart license cost in the model. Default 0 (off).</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="59" t="inlineStr">
         <is>
           <t>Vote Smart Public-Facing Platform License (annual list price)</t>
         </is>
@@ -1930,14 +1947,14 @@
       <c r="B65" s="98" t="n">
         <v>4850</v>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="59" t="inlineStr">
         <is>
           <t>votesmart.org Public-Facing Platform License, 1-year subscription. Quoted June 2026.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="59" t="inlineStr">
         <is>
           <t>Vote Smart applied (toggle x license)</t>
         </is>
@@ -1946,9 +1963,107 @@
         <f>B64*B65</f>
         <v/>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="59" t="inlineStr">
         <is>
           <t>Flows into 'Total other recurring' only when the toggle above = 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="95" t="inlineStr">
+        <is>
+          <t>Crowdfunding (Indiegogo) — one-time raise (added 2026-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Gross campaign goal / raise</t>
+        </is>
+      </c>
+      <c r="B69" s="117" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H69" s="118" t="inlineStr">
+        <is>
+          <t>Indiegogo Flexible-funding goal. Blue = edit me.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Indiegogo platform fee rate</t>
+        </is>
+      </c>
+      <c r="B70" s="119" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H70" s="118" t="inlineStr">
+        <is>
+          <t>Indiegogo flat 5% platform fee (Flexible or Fixed) as of 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Payment processing rate (effective)</t>
+        </is>
+      </c>
+      <c r="B71" s="119" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H71" s="118" t="inlineStr">
+        <is>
+          <t>~2.9% + $0.30 per contribution; ~3% effective at typical gift sizes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Combined Indiegogo fee rate</t>
+        </is>
+      </c>
+      <c r="B72" s="120">
+        <f>B70+B71</f>
+        <v/>
+      </c>
+      <c r="H72" s="118" t="inlineStr">
+        <is>
+          <t>Auto. ~8% all-in — vs GoFundMe's 0% platform / optional-donor-tip model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Net proceeds after fees</t>
+        </is>
+      </c>
+      <c r="B73" s="121">
+        <f>B69*(1-B72)</f>
+        <v/>
+      </c>
+      <c r="H73" s="118" t="inlineStr">
+        <is>
+          <t>What actually lands in the business account. ~$23,000 on a funded $25K raise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>• One-time inflow. Deliberately NOT in 'Total other recurring' (B37) or the 5-Year P&amp;L — those model ongoing operations only. The raise funds the Year-2 buffer; see indiegogo_draft.md.</t>
         </is>
       </c>
     </row>

</xml_diff>